<commit_message>
KPIs reescritos em linguagem natural, com como medir e por que importa, em abas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/07-kpis.xlsx
+++ b/07-kpis.xlsx
@@ -458,10 +458,10 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -474,17 +474,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>KPIs para Topo de Funil</t>
+          <t>KPIs para Topo de funil</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>KPIs para Meio de Funil</t>
+          <t>KPIs para Meio de funil</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>KPIs para Fundo de Funil</t>
+          <t>KPIs para Fundo de funil</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -515,54 +515,68 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="560" customHeight="1">
+    <row r="4" ht="640" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>• Alcance e visualizações dos vídeos
-Mede quantas pessoas do público veem os Reels, TikToks e vídeos no Facebook, por criador parceiro. É o primeiro sinal de que a mensagem chega ao aposentado e ao filho que reserva para ele.
-• Cliques no link do WhatsApp (e custo por clique)
-Mostra quantos curiosos saem da publicação e vão falar com a pousada. Liga o conteúdo ao objetivo de formar a lista de contatos.
-• Visualizações do Google Perfil da Empresa
-O Google é a principal fonte de pesquisa do público. Medir mostra se a correção do perfil traz gente nova.</t>
+          <t>Objetivo da etapa: Ser encontrado por quem procura sossego
+• Alcance dos vídeos
+Como medir: Número de pessoas que viram cada Reels, TikTok e vídeo no Facebook, separado por criador.
+Por que importa: Sem gente vendo o vídeo não existe contato. É o primeiro número que mostra se o criador que a gente pagou está chegando no público certo, e dá para comparar um criador com o outro.
+• Cliques no link do WhatsApp
+Como medir: Cliques no link da bio, no QR code e no botão do Google, cada um com a sua etiqueta de origem.
+Por que importa: Ver o vídeo não paga a conta. O clique mostra quem quis conversar de verdade com a pousada, e liga o conteúdo ao objetivo de formar a lista de contatos.
+• Visitas ao Google Perfil
+Como medir: Relatório do próprio Google Perfil da Empresa: buscas, ligações e pedidos de rota.
+Por que importa: O aposentado pesquisa no Google antes de decidir. Se o perfil corrigido passa a receber mais visitas, a primeira correção do plano está funcionando.</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>• Contatos novos no WhatsApp, por origem
-Conta quem entrou na lista vindo de criador, QR code, excursão ou Google. Acompanha a meta de 300 contatos e mostra qual parceria vale repetir.
-• Tempo da primeira resposta
-Meta de até 15 minutos no horário comercial. O lead esfria rápido e o público idoso quer falar com uma pessoa.
+          <t>Objetivo da etapa: Manter o interesse até a reserva
+• Contatos novos no WhatsApp (Meta: 300 contatos)
+Como medir: Quantas pessoas entram na lista por mês, anotando de onde veio cada uma: criador, QR code, excursão ou Google.
+Por que importa: Chegar a 300 contatos é um dos objetivos. Saber a origem mostra qual parceria vale pagar de novo e qual dá para largar.
+• Tempo da primeira resposta (Meta: até 15 minutos)
+Como medir: Horário da mensagem recebida comparado com o da primeira resposta, no WhatsApp Business, em horário comercial.
+Por que importa: Quem pergunta e fica esperando acaba reservando em outro lugar. Responder rápido é o que mais depende da gente.
 • Respostas às mensagens quinzenais
-Mostra se o contato mantém o interesse sem cansar: quantos respondem, pedem data ou saem da lista.</t>
+Como medir: A cada envio, contar quantos respondem, quantos pedem data e quantos saem da lista.
+Por que importa: Serve para acertar o tom e a frequência sem encher a paciência de ninguém.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>• Taxa de conversão de contato em reserva
-Reservas fechadas divididas pelos contatos recebidos. Diz se a estrutura, o café e a oferta estão convencendo.
-• Percentual de reservas diretas
-Meta de 50%. Cada reserva direta evita a comissão de 15% a 25% das OTAs.
-• Ocupação de domingo a quinta
-Meta de 40%. Mede o objetivo principal do pacote Sossego de Meio de Semana.
-• Custo por reserva
-Soma do investimento (criadores e mídia) dividida pelas reservas. Mostra se a parceria paga se paga.</t>
+          <t>Objetivo da etapa: Fechar a reserva
+• Contato que vira reserva
+Como medir: Reservas fechadas no mês divididas pelos contatos que chegaram no mesmo mês.
+Por que importa: Diz se o quarto, o café e a oferta convencem. Se muita gente pergunta e pouca reserva, o problema está na oferta ou na resposta, e não no vídeo.
+• Reservas diretas (Meta: 50%)
+Como medir: Reservas feitas por WhatsApp, telefone e Instagram divididas pelo total de reservas.
+Por que importa: Cada reserva direta evita a comissão de 15% a 25% das plataformas e deixa o hóspede no nosso contato, pronto para voltar.
+• Ocupação de domingo a quinta (Meta: 40%)
+Como medir: Diárias vendidas de domingo a quinta divididas pelas diárias disponíveis nesses dias.
+Por que importa: É onde a pousada está mais vazia e quando o aposentado consegue viajar. Mede direto o pacote Sossego de Meio de Semana.</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>• Taxa de retorno
-Hóspedes com segunda estadia, incluindo os que usam o Bilhete de Volta. Meta de duas estadias por ano por hóspede, que sustenta o tempo de vida do cliente.
-• Novas avaliações e nota no Google
-O hóspede satisfeito avalia. Meta de manter 4,7 ou mais e somar novas avaliações depois de cada estadia.
+          <t>Objetivo da etapa: Fazer o hóspede voltar e indicar
+• Taxa de retorno (Meta: 2 estadias por ano)
+Como medir: Hóspedes que voltam, incluindo quem usou o Bilhete de Volta, divididos pelos hóspedes do período.
+Por que importa: Segurar um hóspede custa menos que conquistar outro, e é isso que aumenta o tempo de vida do cliente.
+• Avaliações e nota no Google (Meta: nota 4,7 ou mais)
+Como medir: Quantas avaliações novas chegam depois de cada estadia e qual é a nota média.
+Por que importa: A avaliação nova é o que convence o próximo aposentado desconfiado a reservar.
 • Indicações recebidas
-Quantos hóspedes vieram por indicação do programa Traga um amigo. Mede se o presente e o cantinho fotogênico geram boca a boca.</t>
+Como medir: Perguntar na reserva como conheceu a pousada e contar quem veio pelo Traga um amigo.
+Por que importa: Mostra se o presente na chegada e o cantinho de fotos fazem o hóspede falar da pousada para os outros.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Fonte: metas dos objetivos SMART do plano. Linha de base a medir nos primeiros 60 dias, pois não há benchmark público de conversão e custo por reserva para pousadas (diagnóstico de mercado).</t>
+          <t>Observação: não existe número público de conversão e custo por reserva para pousadas. Nos 60 primeiros dias a gente mede a linha de base, e só depois confirma as metas.</t>
         </is>
       </c>
     </row>

</xml_diff>